<commit_message>
Make May comparison reproducible + reference it in the handoff
- backend/scripts/build_may_comparison.py: committed generator for the May 3-way
  spreadsheet (was ephemeral in /tmp). Self-asserts sacred 415.927,84 + live RL
  29.691,61; ruff/mypy clean. Documents the stale-fixture caveat + how to refresh
  _MAY_OVERRIDES from a fresh closing_2026-05.json.
- Handoff: added a 'May proof-of-match artifact' section (NOTA_MAIO + spreadsheet +
  regenerate command + what 'targets/Alvo' means) so a next agent can find and rebuild it.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reference/comparativo/Comparativo_MBC_Maio_2026.xlsx
+++ b/reference/comparativo/Comparativo_MBC_Maio_2026.xlsx
@@ -101,13 +101,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
@@ -550,240 +549,240 @@
           <t>INSTITUCIONAL</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Recebimento (receita de honorários)</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="4" t="n">
         <v>415928</v>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="4" t="n">
         <v>415928</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="4" t="n">
         <v>415927.84</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="4" t="n">
         <v>-0.16</v>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>bate exato</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Sistema reproduz a planilha (diferença ≤ R$1 é só arredondamento).</t>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Sistema reproduz a planilha (diferença ≤ R$1 = arredondamento).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Custos Diretos (custo equipe + comissão)</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="4" t="n">
         <v>210089.46</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="4" t="n">
         <v>210089.46</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="4" t="n">
         <v>210089.45</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="4" t="n">
         <v>-0.01</v>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>bate exato</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Sistema reproduz a planilha (diferença ≤ R$1 é só arredondamento).</t>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Sistema reproduz a planilha (diferença ≤ R$1 = arredondamento).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Despesas Institucionais</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="7" t="n">
         <v>105511.43</v>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="7" t="n">
         <v>105640.6</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="7" t="n">
         <v>105640.6</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="7" t="n">
         <v>129.17</v>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>sistema mais correto</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>Aluguel líquido da sublocação Belline: banco 24.359,77 vs planilha 24.230,60 (+129,17). Renata confirmou: usar o banco.</t>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Aluguel líquido da sublocação Belline: banco 24.359,77 vs planilha 24.230,60 (+129,17). Renata: usar o banco.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Resultado Bruto</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="10" t="n">
         <v>100327.11</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="10" t="n">
         <v>100197.94</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="10" t="n">
         <v>100197.79</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="10" t="n">
         <v>-129.32</v>
       </c>
-      <c r="F6" s="10" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>consequência do aluguel</t>
         </is>
       </c>
-      <c r="G6" s="12" t="inlineStr">
-        <is>
-          <t>Reflete o +129,17 do aluguel na linha de despesas (RB = -129,17).</t>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>Reflete o ±129,17 do aluguel.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Imposto (15% do recebimento)</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="4" t="n">
         <v>62389.2</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="4" t="n">
         <v>62389.2</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="4" t="n">
         <v>62389.18</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="4" t="n">
         <v>-0.02</v>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>bate exato</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Sistema reproduz a planilha (diferença ≤ R$1 é só arredondamento).</t>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Sistema reproduz a planilha (diferença ≤ R$1 = arredondamento).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Amortização</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="4" t="n">
         <v>8117</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="4" t="n">
         <v>8117</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="4" t="n">
         <v>8117</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>bate exato</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Sistema reproduz a planilha (diferença ≤ R$1 é só arredondamento).</t>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Sistema reproduz a planilha (diferença ≤ R$1 = arredondamento).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Resultado Líquido</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="10" t="n">
         <v>29820.91</v>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="10" t="n">
         <v>29691.74</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="10" t="n">
         <v>29691.61</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="10" t="n">
         <v>-129.3</v>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>consequência do aluguel</t>
         </is>
       </c>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>Reflete o +129,17 do aluguel.</t>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>Reflete o ±129,17 do aluguel.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Reserva de Bônus</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="10" t="n">
         <v>2982.09</v>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="10" t="n">
         <v>2969.17</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="10" t="n">
         <v>2969.16</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="10" t="n">
         <v>-12.93</v>
       </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>consequência do aluguel</t>
         </is>
       </c>
-      <c r="G10" s="12" t="inlineStr">
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>10% do líquido corrigido.</t>
         </is>
@@ -795,97 +794,97 @@
           <t>ÁREA — Contencioso</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Recebimento</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="4" t="n">
         <v>240445</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="4" t="n">
         <v>240445</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="4" t="n">
         <v>240444.72</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="4" t="n">
         <v>-0.28</v>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>bate exato</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Sistema reproduz a planilha (diferença ≤ R$1 é só arredondamento).</t>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Sistema reproduz a planilha (diferença ≤ R$1 = arredondamento).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Custo equipe</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="4" t="n">
         <v>74141.21000000001</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="4" t="n">
         <v>74141.21000000001</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="4" t="n">
         <v>74141.21000000001</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>bate exato</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Sistema reproduz a planilha (diferença ≤ R$1 é só arredondamento).</t>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Sistema reproduz a planilha (diferença ≤ R$1 = arredondamento).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Resultado Bruto</t>
         </is>
       </c>
-      <c r="B14" s="11" t="n">
+      <c r="B14" s="10" t="n">
         <v>128472.17</v>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="10" t="n">
         <v>129860.86</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="10" t="n">
         <v>129860.86</v>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="E14" s="10" t="n">
         <v>1388.69</v>
       </c>
-      <c r="F14" s="10" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>regrupamento (Renata)</t>
         </is>
       </c>
-      <c r="G14" s="12" t="inlineStr">
-        <is>
-          <t>Despesas Área alocadas pelo rótulo/centro de custo (fórmula da planilha tinha deslocamento de 1 linha em Viagens). Renata confirmou: alocar pela área do rótulo. Soma das 3 áreas é a mesma.</t>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Despesas Área alocadas pelo rótulo/centro de custo (fórmula da planilha tinha deslocamento de 1 linha em Viagens). Soma das 3 áreas é a mesma.</t>
         </is>
       </c>
     </row>
@@ -895,97 +894,97 @@
           <t>ÁREA — Econômico</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Recebimento</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B16" s="4" t="n">
         <v>166876</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="4" t="n">
         <v>166876</v>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="D16" s="4" t="n">
         <v>166875.57</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="4" t="n">
         <v>-0.43</v>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>bate exato</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Sistema reproduz a planilha (diferença ≤ R$1 é só arredondamento).</t>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Sistema reproduz a planilha (diferença ≤ R$1 = arredondamento).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Custo equipe</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B17" s="4" t="n">
         <v>79436.24000000001</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="4" t="n">
         <v>79436.24000000001</v>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="4" t="n">
         <v>79436.24000000001</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E17" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>bate exato</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>Sistema reproduz a planilha (diferença ≤ R$1 é só arredondamento).</t>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Sistema reproduz a planilha (diferença ≤ R$1 = arredondamento).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Resultado Bruto</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="10" t="n">
         <v>44916.89</v>
       </c>
-      <c r="C18" s="11" t="n">
+      <c r="C18" s="10" t="n">
         <v>43444.15</v>
       </c>
-      <c r="D18" s="11" t="n">
+      <c r="D18" s="10" t="n">
         <v>43444.15</v>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E18" s="10" t="n">
         <v>-1472.74</v>
       </c>
-      <c r="F18" s="10" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>regrupamento (Renata)</t>
         </is>
       </c>
-      <c r="G18" s="12" t="inlineStr">
-        <is>
-          <t>Despesas Área alocadas pelo rótulo/centro de custo (fórmula da planilha tinha deslocamento de 1 linha em Viagens). Renata confirmou: alocar pela área do rótulo. Soma das 3 áreas é a mesma.</t>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>Despesas Área alocadas pelo rótulo/centro de custo (fórmula da planilha tinha deslocamento de 1 linha em Viagens). Soma das 3 áreas é a mesma.</t>
         </is>
       </c>
     </row>
@@ -995,111 +994,111 @@
           <t>ÁREA — Arbitragem</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Recebimento</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B20" s="4" t="n">
         <v>41860</v>
       </c>
-      <c r="C20" s="5" t="n">
+      <c r="C20" s="4" t="n">
         <v>41860</v>
       </c>
-      <c r="D20" s="5" t="n">
+      <c r="D20" s="4" t="n">
         <v>41859.35</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E20" s="4" t="n">
         <v>-0.65</v>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>bate exato</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>Sistema reproduz a planilha (diferença ≤ R$1 é só arredondamento).</t>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Sistema reproduz a planilha (diferença ≤ R$1 = arredondamento).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Custo equipe</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
+      <c r="B21" s="4" t="n">
         <v>54383.94</v>
       </c>
-      <c r="C21" s="5" t="n">
+      <c r="C21" s="4" t="n">
         <v>54383.94</v>
       </c>
-      <c r="D21" s="5" t="n">
+      <c r="D21" s="4" t="n">
         <v>54383.94</v>
       </c>
-      <c r="E21" s="5" t="n">
+      <c r="E21" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>bate exato</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Sistema reproduz a planilha (diferença ≤ R$1 é só arredondamento).</t>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Sistema reproduz a planilha (diferença ≤ R$1 = arredondamento).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Resultado Bruto</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n">
+      <c r="B22" s="10" t="n">
         <v>-39808.95</v>
       </c>
-      <c r="C22" s="11" t="n">
+      <c r="C22" s="10" t="n">
         <v>-39855.42</v>
       </c>
-      <c r="D22" s="11" t="n">
+      <c r="D22" s="10" t="n">
         <v>-39855.42</v>
       </c>
-      <c r="E22" s="11" t="n">
+      <c r="E22" s="10" t="n">
         <v>-46.47</v>
       </c>
-      <c r="F22" s="10" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>regrupamento (Renata)</t>
         </is>
       </c>
-      <c r="G22" s="12" t="inlineStr">
-        <is>
-          <t>Despesas Área alocadas pelo rótulo/centro de custo (fórmula da planilha tinha deslocamento de 1 linha em Viagens). Renata confirmou: alocar pela área do rótulo. Soma das 3 áreas é a mesma.</t>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>Despesas Área alocadas pelo rótulo/centro de custo (fórmula da planilha tinha deslocamento de 1 linha em Viagens). Soma das 3 áreas é a mesma.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Legenda: verde = bate exato · amarelo = banco mais completo/correto · cinza = consequência/arredondamento.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>Recebimento por área usa a base do Demonstrativo por profissional (DB_RESULTADO_PROF), a mesma que vocês usam no LegalDesk.</t>
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Recebimento por área usa a base do Demonstrativo por profissional (DB_RESULTADO_PROF), a mesma do LegalDesk.</t>
         </is>
       </c>
     </row>

</xml_diff>